<commit_message>
feat: complete phase 1 database implementation and tenant auth
</commit_message>
<xml_diff>
--- a/apps/api/test_outputs/dcf_model_test_deal.xlsx
+++ b/apps/api/test_outputs/dcf_model_test_deal.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +119,7 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -504,93 +505,131 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Avg Ebitda Margin</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>0.12</v>
-      </c>
+          <t>Revenue Cagr Override</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tax Rate</t>
+          <t>Avg Ebitda Margin</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Da Percent Rev</t>
+          <t>Latest Ebitda Margin</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cap Ex Percent Rev</t>
+          <t>Terminal Ebitda Margin</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.0925</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nwc Percent Rev</t>
+          <t>Tax Rate</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Base Case</t>
-        </is>
+          <t>Opening Tax Loss Carryforward</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Da Percent Rev</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>WACC</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>0.1246</v>
+          <t>Cap Ex Percent Rev</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0.04</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Nwc Percent Rev</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>0.1246</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Terminal Growth Rate</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B16" s="4" t="n">
         <v>0.025</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>WACC Calculation Breakdown</t>
         </is>
@@ -703,25 +742,25 @@
         <v>250000000000</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>262500000000</v>
+        <v>250000000000</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>274687500000</v>
+        <v>250892857142.86</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>286459821428.57</v>
+        <v>252684948979.59</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>297713600127.55</v>
+        <v>255392287718.66</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>308346228703.54</v>
+        <v>259040748971.78</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>318257357483.29</v>
+        <v>263666476631.99</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>327350424839.96</v>
+        <v>269316472559.82</v>
       </c>
     </row>
     <row r="5">
@@ -738,25 +777,25 @@
         <v>0</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>4.64</v>
+        <v>0.36</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4.29</v>
+        <v>0.71</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>3.93</v>
+        <v>1.07</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>3.57</v>
+        <v>1.43</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>3.21</v>
+        <v>1.79</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>2.86</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="6">
@@ -775,25 +814,25 @@
         <v>30000000000</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>31500000000</v>
+        <v>30000000000</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>32962500000</v>
+        <v>30107142857.14</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>34375178571.43</v>
+        <v>30322193877.55</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>35725632015.31</v>
+        <v>30647074526.24</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>37001547444.42</v>
+        <v>31084889876.61</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>38190882897.99</v>
+        <v>31639977195.84</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>39282050980.79</v>
+        <v>32317976707.18</v>
       </c>
     </row>
     <row r="7">
@@ -840,25 +879,25 @@
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>15750000000</v>
+        <v>12500000000</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>16481250000</v>
+        <v>12544642857.14</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>17187589285.71</v>
+        <v>12634247448.98</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>17862816007.65</v>
+        <v>12769614385.93</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>18500773722.21</v>
+        <v>12952037448.59</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>19095441449</v>
+        <v>13183323831.6</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>19641025490.4</v>
+        <v>13465823627.99</v>
       </c>
     </row>
     <row r="9">
@@ -868,25 +907,25 @@
         </is>
       </c>
       <c r="E9" s="9" t="n">
-        <v>15750000000</v>
+        <v>17500000000</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>16481250000</v>
+        <v>17562500000</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>17187589285.71</v>
+        <v>17687946428.57</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>17862816007.65</v>
+        <v>17877460140.31</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>18500773722.21</v>
+        <v>18132852428.02</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>19095441449</v>
+        <v>18456653364.24</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>19641025490.4</v>
+        <v>18852153079.19</v>
       </c>
     </row>
     <row r="10">
@@ -896,25 +935,25 @@
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3937500000</v>
+        <v>4375000000</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>4120312500</v>
+        <v>4390625000</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4296897321.43</v>
+        <v>4421986607.14</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>4465704001.91</v>
+        <v>4469365035.08</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>4625193430.55</v>
+        <v>4533213107.01</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>4773860362.25</v>
+        <v>4614163341.06</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>4910256372.6</v>
+        <v>4713038269.8</v>
       </c>
     </row>
     <row r="11">
@@ -924,25 +963,25 @@
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>11812500000</v>
+        <v>13125000000</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>12360937500</v>
+        <v>13171875000</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>12890691964.29</v>
+        <v>13265959821.43</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>13397112005.74</v>
+        <v>13408095105.23</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>13875580291.66</v>
+        <v>13599639321.02</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>14321581086.75</v>
+        <v>13842490023.18</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>14730769117.8</v>
+        <v>14139114809.39</v>
       </c>
     </row>
     <row r="12">
@@ -952,25 +991,25 @@
         </is>
       </c>
       <c r="E12" s="9" t="n">
-        <v>15750000000</v>
+        <v>12500000000</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>16481250000</v>
+        <v>12544642857.14</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>17187589285.71</v>
+        <v>12634247448.98</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>17862816007.65</v>
+        <v>12769614385.93</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>18500773722.21</v>
+        <v>12952037448.59</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>19095441449</v>
+        <v>13183323831.6</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19641025490.4</v>
+        <v>13465823627.99</v>
       </c>
     </row>
     <row r="13">
@@ -980,25 +1019,25 @@
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>24281250000</v>
+        <v>10000000000</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>25408593750</v>
+        <v>10035714285.71</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>26497533482.14</v>
+        <v>10107397959.18</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>27538508011.8</v>
+        <v>10215691508.75</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>28522026155.08</v>
+        <v>10361629958.87</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>29438805567.2</v>
+        <v>10546659065.28</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>30279914297.7</v>
+        <v>10772658902.39</v>
       </c>
     </row>
     <row r="14">
@@ -1008,25 +1047,25 @@
         </is>
       </c>
       <c r="E14" s="9" t="n">
-        <v>-5136986301.37</v>
+        <v>5821917808.22</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>1502568493.15</v>
+        <v>110078277.89</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>1451382093.93</v>
+        <v>220942829.19</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>1387452168.37</v>
+        <v>333781488.38</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>1310872016.22</v>
+        <v>449810291.48</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>1221919986.55</v>
+        <v>570295190.98</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>1121063098.77</v>
+        <v>696574840.42</v>
       </c>
     </row>
     <row r="15">
@@ -1036,25 +1075,25 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>8418236301.37</v>
+        <v>9803082191.780001</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>1931025256.85</v>
+        <v>15570725293.54</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>2129365673.92</v>
+        <v>15571866482.04</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>2333967833.23</v>
+        <v>15628236494.04</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>2543455842.58</v>
+        <v>15740236519.26</v>
       </c>
       <c r="J15" s="11" t="n">
-        <v>2756296982</v>
+        <v>15908859598.51</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>2970817211.73</v>
+        <v>16135704694.57</v>
       </c>
     </row>
   </sheetData>
@@ -1068,7 +1107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1137,25 +1176,25 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>8418236301.37</v>
+        <v>9803082191.780001</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>1931025256.85</v>
+        <v>15570725293.54</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>2129365673.92</v>
+        <v>15571866482.04</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>2333967833.23</v>
+        <v>15628236494.04</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>2543455842.58</v>
+        <v>15740236519.26</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>2756296982</v>
+        <v>15908859598.51</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>2970817211.73</v>
+        <v>16135704694.57</v>
       </c>
     </row>
     <row r="5">
@@ -1215,50 +1254,68 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Add: Cash &amp; Equivalents</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="n">
+          <t>Less: Lease Liabilities</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Net Debt</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n">
+          <t>Less: CCPS Liability</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Implied Equity Value</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="n">
-        <v>100000000000</v>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Add: Cash &amp; Equivalents</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Shares Outstanding</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>1</v>
+          <t>Net Debt</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
+          <t>Implied Equity Value</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>100000000000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Shares Outstanding</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
           <t>Implied Share Price</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B19" s="14" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1301,7 +1358,7 @@
     </row>
     <row r="4">
       <c r="B4" s="12">
-        <f>'Valuation'!B17</f>
+        <f>'Valuation'!B19</f>
         <v/>
       </c>
       <c r="C4" s="16" t="n">
@@ -1324,101 +1381,51 @@
       <c r="B5" s="16" t="n">
         <v>0.1046</v>
       </c>
-      <c r="C5" s="12" t="n">
-        <v>33668563287.33677</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>34747354324.76938</v>
-      </c>
-      <c r="E5" s="12" t="n">
-        <v>35961671874.44225</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>37338766575.54582</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>38913719710.71598</v>
-      </c>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="16" t="n">
         <v>0.1146</v>
       </c>
-      <c r="C6" s="12" t="n">
-        <v>30629257859.9888</v>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>31451464971.06073</v>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>32365436268.63622</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>33387441998.54926</v>
-      </c>
-      <c r="G6" s="12" t="n">
-        <v>34537840408.09959</v>
-      </c>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="16" t="n">
         <v>0.1246</v>
       </c>
-      <c r="C7" s="12" t="n">
-        <v>28144240553.7785</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>28784734784.2394</v>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>29489535664.34498</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>30268839808.73233</v>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>31135119862.09148</v>
-      </c>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="16" t="n">
         <v>0.1346</v>
       </c>
-      <c r="C8" s="12" t="n">
-        <v>26074243836.94476</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>26582255242.68457</v>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>27136618054.05757</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>27743979222.1584</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>28412320427.21714</v>
-      </c>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="16" t="n">
         <v>0.1446</v>
       </c>
-      <c r="C9" s="12" t="n">
-        <v>24323004867.82836</v>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>24732077516.17979</v>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>25175353563.22281</v>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>25657309893.60292</v>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>26183240341.71844</v>
-      </c>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>